<commit_message>
Add companion agentic extensions as proposed next-version asks, not a CoSAI SRF v1.0 revision.
Keeps L0-L5 and T1-T5, labels spawn, fail-closed halt, and enforcement planes as independently proposed, and regenerates the knowledge layer so CI stays in lockstep.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tools/vendor-risk/how-to/vendor-risk-workpaper.xlsx
+++ b/tools/vendor-risk/how-to/vendor-risk-workpaper.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Tiers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accountability Split" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attestation Reference" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Bank" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attestation Mapping" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contract Clauses" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFP Questions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Risk Tiers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Accountability Split" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Attestation Reference" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Question Bank" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Attestation Mapping" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Contract Clauses" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="RFP Questions" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Question Bank'!$A$1:$K$38</definedName>
@@ -105,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -148,6 +148,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1225,7 +1228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2244,159 +2247,159 @@
       <c r="K22" s="8" t="inlineStr"/>
     </row>
     <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>5. Data, labeling &amp; retrieval</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>Workforce vetting and background checks</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>SOC 2 +</t>
-        </is>
-      </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Which roles or regions are exempt from screening, and the re-screening cadence.</t>
-        </is>
-      </c>
-      <c r="G23" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H23" s="10" t="inlineStr"/>
-      <c r="I23" s="10" t="inlineStr"/>
-      <c r="J23" s="12" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K23" s="10" t="inlineStr"/>
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>4. Agentic AI &amp; autonomous systems</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>L3, L4</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Agent-PaaS</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Spawn and descendant inventory</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Whether the product can create child agents, whether descendant capabilities are narrower than the parent, whether a live inventory of descendants exists, and whether revoke reaches the full tree.</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="n"/>
+      <c r="I23" s="8" t="n"/>
+      <c r="J23" s="11" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K23" s="8" t="n"/>
     </row>
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>5. Data, labeling &amp; retrieval</t>
+          <t>4. Agentic AI &amp; autonomous systems</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L3, L4</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Agent-PaaS</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Confidential-data controls</t>
+          <t>Fail-closed halt authorization</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>SOC 2 +</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>DLP evidence, GeoIP and embargo restrictions, and penetration-test results for any contractor VDI.</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr"/>
-      <c r="I24" s="8" t="inlineStr"/>
+          <t>For irreversible, financially material, security-control-modifying, physical, or cross-organization actions, the action blocks if the assigned halt authority cannot be reached.</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
       <c r="J24" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K24" s="8" t="inlineStr"/>
+      <c r="K24" s="8" t="n"/>
     </row>
     <row r="25" ht="42" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>5. Data, labeling &amp; retrieval</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>Annotation QA and accuracy</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>ISO 9001 +</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>QA methodology documentation and the prior-quarter metrics dashboard.</t>
-        </is>
-      </c>
-      <c r="G25" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H25" s="10" t="inlineStr"/>
-      <c r="I25" s="10" t="inlineStr"/>
-      <c r="J25" s="12" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K25" s="10" t="inlineStr"/>
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>4. Agentic AI &amp; autonomous systems</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>L3, L4</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Agent-PaaS</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Spend ceiling halt vs alert</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Whether the spend or economic ceiling stops the agent or only alerts, and which party owns that control.</t>
+        </is>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="n"/>
     </row>
     <row r="26" ht="42" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>5. Data, labeling &amp; retrieval</t>
+          <t>4. Agentic AI &amp; autonomous systems</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L3, L4</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Agent-PaaS</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Sub-processors and cross-border flow</t>
+          <t>Persistence scope of memory and RAG</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -2406,97 +2409,97 @@
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>Sub-processor list with change control, a data-flow diagram with geographies, audit results, and opt-out.</t>
-        </is>
-      </c>
-      <c r="G26" s="11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H26" s="8" t="inlineStr"/>
-      <c r="I26" s="8" t="inlineStr"/>
+          <t>Whether retained state is request-scoped, handle-scoped, or durable, and who governs durable state.</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="n"/>
+      <c r="I26" s="8" t="n"/>
       <c r="J26" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K26" s="8" t="inlineStr"/>
+      <c r="K26" s="8" t="n"/>
     </row>
     <row r="27" ht="42" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>5. Data, labeling &amp; retrieval</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>Retention and secure deletion</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
-        <is>
-          <t>SOC 2 +</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>Whether you can define the retention policy, plus certificates of data deletion or destruction.</t>
-        </is>
-      </c>
-      <c r="G27" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H27" s="10" t="inlineStr"/>
-      <c r="I27" s="10" t="inlineStr"/>
-      <c r="J27" s="12" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K27" s="10" t="inlineStr"/>
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>4. Agentic AI &amp; autonomous systems</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>L3, L4</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Agent-PaaS</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Enforcement-plane control</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Which plane the vendor actually enforces: north-south (model provider), east-west (agent to agent), or agent-to-tool.</t>
+        </is>
+      </c>
+      <c r="G27" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="n"/>
+      <c r="I27" s="8" t="n"/>
+      <c r="J27" s="11" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K27" s="8" t="n"/>
     </row>
     <row r="28" ht="42" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>5. Data, labeling &amp; retrieval</t>
+          <t>4. Agentic AI &amp; autonomous systems</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L3, L4</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Agent-PaaS</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Retrieval and RAG integrity</t>
+          <t>Owner-of-record vs halt-authority coverage</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>ISO 27001</t>
+          <t>Disclosure</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>Access controls on the vector store, data-poisoning defenses, and tenant isolation of embeddings.</t>
+          <t>Named operational owner coverage and named halt-authority coverage, auditable as two lists.</t>
         </is>
       </c>
       <c r="G28" s="13" t="inlineStr">
@@ -2504,24 +2507,24 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H28" s="8" t="inlineStr"/>
-      <c r="I28" s="8" t="inlineStr"/>
+      <c r="H28" s="8" t="n"/>
+      <c r="I28" s="8" t="n"/>
       <c r="J28" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="K28" s="8" t="inlineStr"/>
+      <c r="K28" s="8" t="n"/>
     </row>
     <row r="29" ht="42" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>6. Consulting &amp; professional services</t>
+          <t>5. Data, labeling &amp; retrieval</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>L1, cross</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -2531,17 +2534,17 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Scope, SLAs, and success KPIs</t>
+          <t>Workforce vetting and background checks</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>SOC 2 +</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>Examples of AI KPI dashboards and prior-project scorecards.</t>
+          <t>Which roles or regions are exempt from screening, and the re-screening cadence.</t>
         </is>
       </c>
       <c r="G29" s="12" t="inlineStr">
@@ -2561,12 +2564,12 @@
     <row r="30" ht="42" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>6. Consulting &amp; professional services</t>
+          <t>5. Data, labeling &amp; retrieval</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>L1, cross</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
@@ -2576,7 +2579,7 @@
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Access controls in client environments</t>
+          <t>Confidential-data controls</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -2586,7 +2589,7 @@
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>Restricted data and system-access requirements such as VPN, VDI, Jupyter Hub, and IDE.</t>
+          <t>DLP evidence, GeoIP and embargo restrictions, and penetration-test results for any contractor VDI.</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr">
@@ -2606,12 +2609,12 @@
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>6. Consulting &amp; professional services</t>
+          <t>5. Data, labeling &amp; retrieval</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>L1, cross</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
@@ -2621,17 +2624,17 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Ownership of code and models produced</t>
+          <t>Annotation QA and accuracy</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>ISO 9001 +</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>Contracts addressing IP or joint ownership, plus SBOM and AIBOM breakdowns of what was delivered.</t>
+          <t>QA methodology documentation and the prior-quarter metrics dashboard.</t>
         </is>
       </c>
       <c r="G31" s="12" t="inlineStr">
@@ -2651,12 +2654,12 @@
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>6. Consulting &amp; professional services</t>
+          <t>5. Data, labeling &amp; retrieval</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>L1, cross</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -2666,17 +2669,17 @@
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Security posture of the firm</t>
+          <t>Sub-processors and cross-border flow</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>SOC 2 / ISO 27001</t>
+          <t>Disclosure</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>Third-party attestation results for the consulting firm itself.</t>
+          <t>Sub-processor list with change control, a data-flow diagram with geographies, audit results, and opt-out.</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr">
@@ -2696,12 +2699,12 @@
     <row r="33" ht="42" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>6. Consulting &amp; professional services</t>
+          <t>5. Data, labeling &amp; retrieval</t>
         </is>
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>L1, cross</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -2711,7 +2714,7 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>Post-engagement data destruction</t>
+          <t>Retention and secure deletion</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
@@ -2721,7 +2724,7 @@
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>Destruction certificates, IDE and repo sanitization process, and developer workstation and VDI cache wipe.</t>
+          <t>Whether you can define the retention policy, plus certificates of data deletion or destruction.</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr">
@@ -2741,37 +2744,37 @@
     <row r="34" ht="42" customHeight="1">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>7. Software, VARs &amp; distributors</t>
+          <t>5. Data, labeling &amp; retrieval</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>L3, L4</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Patch and update responsibility</t>
+          <t>Retrieval and RAG integrity</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>ISO 27001</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>Model, dataset, and tool patch schedule, plus an end-of-life matrix by product.</t>
-        </is>
-      </c>
-      <c r="G34" s="11" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Access controls on the vector store, data-poisoning defenses, and tenant isolation of embeddings.</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr"/>
@@ -2786,32 +2789,32 @@
     <row r="35" ht="42" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>7. Software, VARs &amp; distributors</t>
+          <t>6. Consulting &amp; professional services</t>
         </is>
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>L3, L4</t>
+          <t>L1, cross</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>Reseller controls aligned to OEM</t>
+          <t>Scope, SLAs, and success KPIs</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>Disclosure</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>A controls-hardening benchmark and a clause ensuring the vendor cannot weaken security settings over time.</t>
+          <t>Examples of AI KPI dashboards and prior-project scorecards.</t>
         </is>
       </c>
       <c r="G35" s="12" t="inlineStr">
@@ -2831,32 +2834,32 @@
     <row r="36" ht="42" customHeight="1">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>7. Software, VARs &amp; distributors</t>
+          <t>6. Consulting &amp; professional services</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>L3, L4</t>
+          <t>L1, cross</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Support and escalation path</t>
+          <t>Access controls in client environments</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>Contract</t>
+          <t>SOC 2 +</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>Named contacts and numbers, and the incident-response process.</t>
+          <t>Restricted data and system-access requirements such as VPN, VDI, Jupyter Hub, and IDE.</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr">
@@ -2876,32 +2879,32 @@
     <row r="37" ht="42" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>7. Software, VARs &amp; distributors</t>
+          <t>6. Consulting &amp; professional services</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>L3, L4</t>
+          <t>L1, cross</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>Downstream supply-chain vetting</t>
+          <t>Ownership of code and models produced</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>Disclosure</t>
+          <t>Contract</t>
         </is>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>Current sub-provider inventory with geographic locations and data roles, audit results, and opt-out options.</t>
+          <t>Contracts addressing IP or joint ownership, plus SBOM and AIBOM breakdowns of what was delivered.</t>
         </is>
       </c>
       <c r="G37" s="12" t="inlineStr">
@@ -2921,32 +2924,32 @@
     <row r="38" ht="42" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>7. Software, VARs &amp; distributors</t>
+          <t>6. Consulting &amp; professional services</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>L3, L4</t>
+          <t>L1, cross</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Licensing terms and warranty</t>
+          <t>Security posture of the firm</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>Legal review</t>
+          <t>SOC 2 / ISO 27001</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>Licensing and warranty coverage, with legal sign-off.</t>
+          <t>Third-party attestation results for the consulting firm itself.</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr">
@@ -2963,10 +2966,280 @@
       </c>
       <c r="K38" s="8" t="inlineStr"/>
     </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>6. Consulting &amp; professional services</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>L1, cross</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Post-engagement data destruction</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>SOC 2 +</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Destruction certificates, IDE and repo sanitization process, and developer workstation and VDI cache wipe.</t>
+        </is>
+      </c>
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H39" s="10" t="inlineStr"/>
+      <c r="I39" s="10" t="inlineStr"/>
+      <c r="J39" s="12" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K39" s="10" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>7. Software, VARs &amp; distributors</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>L3, L4</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>varies</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Patch and update responsibility</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Model, dataset, and tool patch schedule, plus an end-of-life matrix by product.</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr"/>
+      <c r="I40" s="8" t="inlineStr"/>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K40" s="8" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>7. Software, VARs &amp; distributors</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>L3, L4</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>varies</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Reseller controls aligned to OEM</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>A controls-hardening benchmark and a clause ensuring the vendor cannot weaken security settings over time.</t>
+        </is>
+      </c>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" s="10" t="inlineStr"/>
+      <c r="I41" s="10" t="inlineStr"/>
+      <c r="J41" s="12" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K41" s="10" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>7. Software, VARs &amp; distributors</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>L3, L4</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>varies</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Support and escalation path</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>Named contacts and numbers, and the incident-response process.</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr"/>
+      <c r="I42" s="8" t="inlineStr"/>
+      <c r="J42" s="11" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K42" s="8" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>7. Software, VARs &amp; distributors</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>L3, L4</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>varies</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Downstream supply-chain vetting</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>Current sub-provider inventory with geographic locations and data roles, audit results, and opt-out options.</t>
+        </is>
+      </c>
+      <c r="G43" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" s="10" t="inlineStr"/>
+      <c r="I43" s="10" t="inlineStr"/>
+      <c r="J43" s="12" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K43" s="10" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>7. Software, VARs &amp; distributors</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>L3, L4</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>varies</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Licensing terms and warranty</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Legal review</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>Licensing and warranty coverage, with legal sign-off.</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr"/>
+      <c r="I44" s="8" t="inlineStr"/>
+      <c r="J44" s="11" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="K44" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K38"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Partial,N/A,Not Started"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3210,7 +3483,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>For any autonomous or agentic capability, Vendor shall provide [Customer] with configurable controls over autonomy level and human override, scope and rate limits on tool and action use, the ability to require human approval for [defined high-impact actions], a complete audit trail of agent actions, and a documented mechanism to immediately suspend agent activity. Vendor shall not change default autonomy or override settings without prior written notice.</t>
+          <t>For any autonomous or agentic capability, Vendor shall provide [Customer] with configurable controls over autonomy level and human override, scope and rate limits on tool and action use, the ability to require human approval for [defined high-impact actions], a complete audit trail of agent actions, and a documented mechanism to immediately suspend agent activity. High-impact actions that are irreversible, financially material, security-control-modifying, physical, or cross-organizational shall fail closed if the assigned halt authority cannot be reached. If the product can spawn child agents, descendant capabilities shall not exceed the parent, a live descendant inventory shall be available, and revocation shall reach the full tree. A spend or economic ceiling shall halt the agent, not only alert, unless [Customer] has accepted alert-only in writing. Vendor shall not change default autonomy or override settings without prior written notice.</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3263,114 +3536,169 @@
       </c>
     </row>
     <row r="2" ht="38" customHeight="1">
-      <c r="A2" s="15" t="n">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Which SRF layers does your offering touch (L1 to L5), and what is your operating model (AI-SaaS, AI-PaaS, Agent-PaaS, IaaS)?</t>
         </is>
       </c>
-      <c r="C2" s="16" t="inlineStr"/>
+      <c r="C2" s="4" t="n"/>
     </row>
     <row r="3" ht="38" customHeight="1">
-      <c r="A3" s="14" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>Provide a responsibility matrix stating which controls you own and which remain with us.</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr"/>
+      <c r="C3" s="4" t="n"/>
     </row>
     <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="15" t="n">
+      <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>List the foundation models and sub-processors behind the service, with their geographic locations and data roles.</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr"/>
+      <c r="C4" s="4" t="n"/>
     </row>
     <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="14" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Confirm in writing that our data, prompts, and outputs are not used to train shared models, and describe how this is enforced.</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr"/>
+      <c r="C5" s="4" t="n"/>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="15" t="n">
+      <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Provide your current attestations (SOC 2 Type II, ISO/IEC 27001, ISO/IEC 42001) and, for AI governance, your ISO 42001 certification or NIST AI RMF profile.</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr"/>
+      <c r="C6" s="4" t="n"/>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="14" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Describe your defenses against prompt injection, including indirect injection from retrieved content or tool output.</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr"/>
+      <c r="C7" s="4" t="n"/>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="15" t="n">
+      <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Provide model and weight provenance, signing, and an AI bill of materials (AIBOM).</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr"/>
+      <c r="C8" s="4" t="n"/>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="14" t="n">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>For agentic features, state the autonomy levels and human-override tiers supported, the permission model, and the kill-switch mechanism.</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr"/>
+      <c r="C9" s="4" t="n"/>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="15" t="n">
+      <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>State whether the product can spawn child agents, how descendant authority is narrowed, how descendants are inventoried, and how revoke reaches the tree.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>For high-impact actions, confirm fail-closed behavior when halt authority is unreachable, and whether spend ceilings halt or only alert.</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>State persistence scope of memory and RAG (request, handle-scoped, or durable) and who governs durable state.</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>State which enforcement plane the vendor actually controls (north-south, east-west, or agent-to-tool).</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Name operational owner coverage and halt-authority coverage as two auditable lists.</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>Describe how you notify customers of model, sub-processor, and autonomy changes, and the notice period.</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr"/>
-    </row>
-    <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="C15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>Provide your data-retention and secure-deletion policy, including certificates of destruction on exit.</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr"/>
+      <c r="C16" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>